<commit_message>
added some formatting and cleaned the codebase
</commit_message>
<xml_diff>
--- a/100048497/output.xlsx
+++ b/100048497/output.xlsx
@@ -1,19 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carla\clariant\mini_project\100048497\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E9BAE6-0225-4646-9789-4DD604255D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="2895" yWindow="1620" windowWidth="23985" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="200127802" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="bin_200127802">200127802!$K$2:INDEX(200127802!$K:$K,2+COUNT(_xlfn.ANCHORARRAY(200127802!$K$2))-1)</definedName>
-    <definedName name="frequencies_200127802">200127802!$M$2:INDEX(200127802!$M:$M,2+COUNT(_xlfn.ANCHORARRAY(200127802!$M$2))-1)</definedName>
+    <definedName name="bin_200127802">'200127802'!$K$2:INDEX('200127802'!$K:$K,2+COUNT(_xlfn.ANCHORARRAY('200127802'!$K$2))-1)</definedName>
+    <definedName name="frequencies_200127802">'200127802'!$M$2:INDEX('200127802'!$M:$M,2+COUNT(_xlfn.ANCHORARRAY('200127802'!$M$2))-1)</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -87,8 +106,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -151,12 +170,30 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
   <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
   <c:chart>
     <c:title>
       <c:tx>
@@ -174,46 +211,94 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
+      <c:overlay val="0"/>
     </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:invertIfNegative val="0"/>
           <c:cat>
-            <c:strRef>
-              <c:f>200127802!bin_200127802</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
+            <c:numRef>
+              <c:f>[0]!bin_200127802</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>Particle</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>200127802!frequencies_200127802</c:f>
+              <c:f>[0]!frequencies_200127802</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>181</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>54</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-193C-4A39-9694-8274D33B90B5}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
         <c:gapWidth val="0"/>
         <c:axId val="50010001"/>
         <c:axId val="50010002"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
@@ -228,31 +313,76 @@
             <c:symbol val="none"/>
           </c:marker>
           <c:cat>
-            <c:strRef>
-              <c:f>200127802!bin_200127802</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
+            <c:numRef>
+              <c:f>[0]!bin_200127802</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>Particle</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>200127802!frequencies_200127802</c:f>
+              <c:f>[0]!frequencies_200127802</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>181</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>54</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-193C-4A39-9694-8274D33B90B5}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
         <c:marker val="1"/>
+        <c:smooth val="0"/>
         <c:axId val="50010001"/>
         <c:axId val="50010002"/>
       </c:lineChart>
@@ -261,6 +391,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
+        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:title>
           <c:tx>
@@ -278,15 +409,18 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
+          <c:overlay val="0"/>
         </c:title>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50010002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="50010002"/>
@@ -294,6 +428,7 @@
           <c:orientation val="minMax"/>
           <c:min val="0"/>
         </c:scaling>
+        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:title>
           <c:tx>
@@ -311,10 +446,11 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
+          <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50010001"/>
         <c:crosses val="autoZero"/>
@@ -322,6 +458,8 @@
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -348,7 +486,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -367,9 +511,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -407,7 +551,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -441,6 +585,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -475,9 +620,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -650,11 +796,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R301"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -698,12 +850,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>2.565</v>
+        <v>2.5649999999999999</v>
       </c>
       <c r="E2">
         <v>1.153</v>
@@ -712,148 +864,208 @@
         <v>5.04</v>
       </c>
       <c r="G2">
-        <v>2.491713333333333</v>
+        <v>2.4917133333333328</v>
       </c>
       <c r="H2">
-        <v>0.5832736736875285</v>
+        <v>0.58327367368752847</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2" cm="1">
-        <f t="array" ref="K2">_xlfn.SEQUENCE(INT((P2-O2)/J2)+1,1,O2,J2)</f>
-        <v>0</v>
+        <f t="array" ref="K2:K7">_xlfn.SEQUENCE(INT((P2-O2)/J2)+1,1,O2,J2)</f>
+        <v>1</v>
       </c>
       <c r="L2" cm="1">
-        <f t="array" ref="L2">(_xlfn.ANCHORARRAY(Q2)+_xlfn.ANCHORARRAY(K2))/2</f>
-        <v>0</v>
+        <f t="array" ref="L2:L7">(_xlfn.ANCHORARRAY(Q2)+_xlfn.ANCHORARRAY(K2))/2</f>
+        <v>1.5</v>
       </c>
       <c r="M2" cm="1">
-        <f t="array" ref="M2">COUNTIFS(B2:B301, "&gt;="&amp;(_xlfn.ANCHORARRAY(K2)-$J$2), B2:B301, "&lt;"&amp;_xlfn.ANCHORARRAY(K2))</f>
+        <f t="array" ref="M2:M7">COUNTIFS(B2:B301, "&gt;="&amp;(_xlfn.ANCHORARRAY(K2)-$J$2), B2:B301, "&lt;"&amp;_xlfn.ANCHORARRAY(K2))</f>
         <v>0</v>
       </c>
       <c r="O2">
         <f>FLOOR(E2,J2)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P2">
         <f>CEILING(F2,J2)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q2" cm="1">
-        <f t="array" ref="Q2">_xlfn.SEQUENCE(INT((P2-O2)/J2)+1,1,O2+J2,J2)</f>
-        <v>0</v>
+        <f t="array" ref="Q2:Q7">_xlfn.SEQUENCE(INT((P2-O2)/J2)+1,1,O2+J2,J2)</f>
+        <v>2</v>
       </c>
       <c r="R2" cm="1">
         <f t="array" ref="R2">ROWS(_xlfn.ANCHORARRAY(K2))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1.588</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18">
+        <v>1.5880000000000001</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <v>2.5</v>
+      </c>
+      <c r="M3">
+        <v>63</v>
+      </c>
+      <c r="Q3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>3.053</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18">
+        <v>3.0529999999999999</v>
+      </c>
+      <c r="K4">
+        <v>3</v>
+      </c>
+      <c r="L4">
+        <v>3.5</v>
+      </c>
+      <c r="M4">
+        <v>181</v>
+      </c>
+      <c r="Q4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5">
-        <v>1.941</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18">
+        <v>1.9410000000000001</v>
+      </c>
+      <c r="K5">
+        <v>4</v>
+      </c>
+      <c r="L5">
+        <v>4.5</v>
+      </c>
+      <c r="M5">
+        <v>54</v>
+      </c>
+      <c r="Q5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
-        <v>2.406</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18">
+        <v>2.4060000000000001</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
+        <v>5.5</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+      <c r="Q6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>2.565</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18">
+        <v>2.5649999999999999</v>
+      </c>
+      <c r="K7">
+        <v>6</v>
+      </c>
+      <c r="L7">
+        <v>6.5</v>
+      </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
+      <c r="Q7">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8">
-        <v>1.832</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18">
+        <v>1.8320000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>1.896</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18">
+        <v>1.8959999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10">
-        <v>2.245</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18">
+        <v>2.2450000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11">
-        <v>2.667</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18">
+        <v>2.6669999999999998</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12">
-        <v>2.038</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18">
+        <v>2.0379999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13">
-        <v>2.642</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18">
+        <v>2.6419999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14">
-        <v>1.749</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18">
+        <v>1.7490000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15">
-        <v>2.598</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18">
+        <v>2.5979999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -861,31 +1073,31 @@
         <v>2.242</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17">
-        <v>2.983</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
+        <v>2.9830000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18">
-        <v>2.281</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
+        <v>2.2810000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19">
-        <v>2.951</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
+        <v>2.9510000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -893,15 +1105,15 @@
         <v>2.359</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21">
-        <v>3.454</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
+        <v>3.4540000000000002</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -909,15 +1121,15 @@
         <v>2.202</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23">
-        <v>2.941</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
+        <v>2.9409999999999998</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -925,15 +1137,15 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25">
-        <v>2.518</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2">
+        <v>2.5179999999999998</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -941,23 +1153,23 @@
         <v>2.073</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27">
-        <v>2.705</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2">
+        <v>2.7050000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28">
-        <v>3.288</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2">
+        <v>3.2879999999999998</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -965,39 +1177,39 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30">
-        <v>2.486</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2">
+        <v>2.4860000000000002</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31">
-        <v>2.038</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2">
+        <v>2.0379999999999998</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32">
-        <v>1.846</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2">
+        <v>1.8460000000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33">
-        <v>2.159</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2">
+        <v>2.1589999999999998</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1005,39 +1217,39 @@
         <v>2.528</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35">
-        <v>2.769</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2">
+        <v>2.7690000000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36">
-        <v>2.667</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2">
+        <v>2.6669999999999998</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37">
-        <v>2.518</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2">
+        <v>2.5179999999999998</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38">
-        <v>2.47</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2">
+        <v>2.4700000000000002</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1045,15 +1257,15 @@
         <v>2.851</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40">
-        <v>3.058</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2">
+        <v>3.0579999999999998</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1061,39 +1273,39 @@
         <v>3.048</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42">
-        <v>3.134</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2">
+        <v>3.1339999999999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43">
-        <v>2.3</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44">
-        <v>2.898</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2">
+        <v>2.8980000000000001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45">
-        <v>2.978</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2">
+        <v>2.9780000000000002</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1101,15 +1313,15 @@
         <v>2.278</v>
       </c>
     </row>
-    <row r="47" spans="1:2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47">
-        <v>1.658</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2">
+        <v>1.6579999999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1117,7 +1329,7 @@
         <v>1.99</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1125,15 +1337,15 @@
         <v>1.234</v>
       </c>
     </row>
-    <row r="50" spans="1:2">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50">
-        <v>2.572</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2">
+        <v>2.5720000000000001</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1141,7 +1353,7 @@
         <v>1.883</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1149,31 +1361,31 @@
         <v>1.746</v>
       </c>
     </row>
-    <row r="53" spans="1:2">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53">
-        <v>3.179</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2">
+        <v>3.1789999999999998</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
       <c r="B54">
-        <v>2.155</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2">
+        <v>2.1549999999999998</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
       <c r="B55">
-        <v>1.293</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2">
+        <v>1.2929999999999999</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1181,15 +1393,15 @@
         <v>1.528</v>
       </c>
     </row>
-    <row r="57" spans="1:2">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
       <c r="B57">
-        <v>2.429</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2">
+        <v>2.4289999999999998</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -1197,7 +1409,7 @@
         <v>1.819</v>
       </c>
     </row>
-    <row r="59" spans="1:2">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -1205,23 +1417,23 @@
         <v>2.044</v>
       </c>
     </row>
-    <row r="60" spans="1:2">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
       <c r="B60">
-        <v>2.751</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2">
+        <v>2.7509999999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
       <c r="B61">
-        <v>2.506</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2">
+        <v>2.5059999999999998</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -1229,7 +1441,7 @@
         <v>1.506</v>
       </c>
     </row>
-    <row r="63" spans="1:2">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -1237,23 +1449,23 @@
         <v>1.819</v>
       </c>
     </row>
-    <row r="64" spans="1:2">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
       <c r="B64">
-        <v>1.293</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2">
+        <v>1.2929999999999999</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
       <c r="B65">
-        <v>1.638</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2">
+        <v>1.6379999999999999</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -1261,7 +1473,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="67" spans="1:2">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -1269,23 +1481,23 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="68" spans="1:2">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
       <c r="B68">
-        <v>1.983</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2">
+        <v>1.9830000000000001</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
       <c r="B69">
-        <v>2.678</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2">
+        <v>2.6779999999999999</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -1293,7 +1505,7 @@
         <v>1.506</v>
       </c>
     </row>
-    <row r="71" spans="1:2">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -1301,7 +1513,7 @@
         <v>1.893</v>
       </c>
     </row>
-    <row r="72" spans="1:2">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -1309,7 +1521,7 @@
         <v>2.7</v>
       </c>
     </row>
-    <row r="73" spans="1:2">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -1317,31 +1529,31 @@
         <v>1.645</v>
       </c>
     </row>
-    <row r="74" spans="1:2">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
       <c r="B74">
-        <v>1.763</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2">
+        <v>1.7629999999999999</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
       <c r="B75">
-        <v>2.075</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2">
+        <v>2.0750000000000002</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
       <c r="B76">
-        <v>2.049</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2">
+        <v>2.0489999999999999</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -1349,23 +1561,23 @@
         <v>3.28</v>
       </c>
     </row>
-    <row r="78" spans="1:2">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
       <c r="B78">
-        <v>1.711</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2">
+        <v>1.7110000000000001</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
       <c r="B79">
-        <v>2.457</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2">
+        <v>2.4569999999999999</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -1373,15 +1585,15 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="81" spans="1:2">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
       <c r="B81">
-        <v>2.078</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2">
+        <v>2.0779999999999998</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -1389,7 +1601,7 @@
         <v>2.411</v>
       </c>
     </row>
-    <row r="83" spans="1:2">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -1397,7 +1609,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="84" spans="1:2">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -1405,7 +1617,7 @@
         <v>2.613</v>
       </c>
     </row>
-    <row r="85" spans="1:2">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -1413,47 +1625,47 @@
         <v>2.851</v>
       </c>
     </row>
-    <row r="86" spans="1:2">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
       <c r="B86">
-        <v>2.898</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2">
+        <v>2.8980000000000001</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
       <c r="B87">
-        <v>3.676</v>
-      </c>
-    </row>
-    <row r="88" spans="1:2">
+        <v>3.6760000000000002</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
       <c r="B88">
-        <v>4.495</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2">
+        <v>4.4950000000000001</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
       <c r="B89">
-        <v>3.131</v>
-      </c>
-    </row>
-    <row r="90" spans="1:2">
+        <v>3.1309999999999998</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
       <c r="B90">
-        <v>3.019</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2">
+        <v>3.0190000000000001</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -1461,23 +1673,23 @@
         <v>3.093</v>
       </c>
     </row>
-    <row r="92" spans="1:2">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
       <c r="B92">
-        <v>2.408</v>
-      </c>
-    </row>
-    <row r="93" spans="1:2">
+        <v>2.4079999999999999</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
       <c r="B93">
-        <v>2.579</v>
-      </c>
-    </row>
-    <row r="94" spans="1:2">
+        <v>2.5790000000000002</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
@@ -1485,15 +1697,15 @@
         <v>1.698</v>
       </c>
     </row>
-    <row r="95" spans="1:2">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
       <c r="B95">
-        <v>2.352</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2">
+        <v>2.3519999999999999</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -1501,7 +1713,7 @@
         <v>2.851</v>
       </c>
     </row>
-    <row r="97" spans="1:2">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
@@ -1509,31 +1721,31 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="98" spans="1:2">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
       <c r="B98">
-        <v>1.933</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2">
+        <v>1.9330000000000001</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
       <c r="B99">
-        <v>3.458</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2">
+        <v>3.4580000000000002</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
       <c r="B100">
-        <v>2.408</v>
-      </c>
-    </row>
-    <row r="101" spans="1:2">
+        <v>2.4079999999999999</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
@@ -1541,7 +1753,7 @@
         <v>3.423</v>
       </c>
     </row>
-    <row r="102" spans="1:2">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>101</v>
       </c>
@@ -1549,23 +1761,23 @@
         <v>3.339</v>
       </c>
     </row>
-    <row r="103" spans="1:2">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
       <c r="B103">
-        <v>1.862</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2">
+        <v>1.8620000000000001</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
       <c r="B104">
-        <v>2.445</v>
-      </c>
-    </row>
-    <row r="105" spans="1:2">
+        <v>2.4449999999999998</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
@@ -1573,7 +1785,7 @@
         <v>1.431</v>
       </c>
     </row>
-    <row r="106" spans="1:2">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
@@ -1581,7 +1793,7 @@
         <v>2.734</v>
       </c>
     </row>
-    <row r="107" spans="1:2">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
       </c>
@@ -1589,23 +1801,23 @@
         <v>2.734</v>
       </c>
     </row>
-    <row r="108" spans="1:2">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>107</v>
       </c>
       <c r="B108">
-        <v>2.916</v>
-      </c>
-    </row>
-    <row r="109" spans="1:2">
+        <v>2.9159999999999999</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>108</v>
       </c>
       <c r="B109">
-        <v>2.457</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2">
+        <v>2.4569999999999999</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>109</v>
       </c>
@@ -1613,15 +1825,15 @@
         <v>3.024</v>
       </c>
     </row>
-    <row r="111" spans="1:2">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>110</v>
       </c>
       <c r="B111">
-        <v>2.078</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2">
+        <v>2.0779999999999998</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>111</v>
       </c>
@@ -1629,7 +1841,7 @@
         <v>2.645</v>
       </c>
     </row>
-    <row r="113" spans="1:2">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
@@ -1637,15 +1849,15 @@
         <v>1.153</v>
       </c>
     </row>
-    <row r="114" spans="1:2">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>113</v>
       </c>
       <c r="B114">
-        <v>1.805</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2">
+        <v>1.8049999999999999</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>114</v>
       </c>
@@ -1653,39 +1865,39 @@
         <v>2.645</v>
       </c>
     </row>
-    <row r="116" spans="1:2">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
       <c r="B116">
-        <v>2.297</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2">
+        <v>2.2970000000000002</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>116</v>
       </c>
       <c r="B117">
-        <v>2.082</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2">
+        <v>2.0819999999999999</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>117</v>
       </c>
       <c r="B118">
-        <v>1.817</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2">
+        <v>1.8169999999999999</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>118</v>
       </c>
       <c r="B119">
-        <v>2.166</v>
-      </c>
-    </row>
-    <row r="120" spans="1:2">
+        <v>2.1659999999999999</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>119</v>
       </c>
@@ -1693,7 +1905,7 @@
         <v>1.153</v>
       </c>
     </row>
-    <row r="121" spans="1:2">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>120</v>
       </c>
@@ -1701,15 +1913,15 @@
         <v>2.089</v>
       </c>
     </row>
-    <row r="122" spans="1:2">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>121</v>
       </c>
       <c r="B122">
-        <v>2.939</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2">
+        <v>2.9390000000000001</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>122</v>
       </c>
@@ -1717,71 +1929,71 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="124" spans="1:2">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>123</v>
       </c>
       <c r="B124">
-        <v>1.866</v>
-      </c>
-    </row>
-    <row r="125" spans="1:2">
+        <v>1.8660000000000001</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>124</v>
       </c>
       <c r="B125">
-        <v>1.898</v>
-      </c>
-    </row>
-    <row r="126" spans="1:2">
+        <v>1.8979999999999999</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>125</v>
       </c>
       <c r="B126">
-        <v>1.834</v>
-      </c>
-    </row>
-    <row r="127" spans="1:2">
+        <v>1.8340000000000001</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>126</v>
       </c>
       <c r="B127">
-        <v>2.517</v>
-      </c>
-    </row>
-    <row r="128" spans="1:2">
+        <v>2.5169999999999999</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>127</v>
       </c>
       <c r="B128">
-        <v>1.703</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2">
+        <v>1.7030000000000001</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>128</v>
       </c>
       <c r="B129">
-        <v>2.078</v>
-      </c>
-    </row>
-    <row r="130" spans="1:2">
+        <v>2.0779999999999998</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>129</v>
       </c>
       <c r="B130">
-        <v>2.326</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2">
+        <v>2.3260000000000001</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>130</v>
       </c>
       <c r="B131">
-        <v>1.467</v>
-      </c>
-    </row>
-    <row r="132" spans="1:2">
+        <v>1.4670000000000001</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>131</v>
       </c>
@@ -1789,7 +2001,7 @@
         <v>1.99</v>
       </c>
     </row>
-    <row r="133" spans="1:2">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>132</v>
       </c>
@@ -1797,15 +2009,15 @@
         <v>2.093</v>
       </c>
     </row>
-    <row r="134" spans="1:2">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>133</v>
       </c>
       <c r="B134">
-        <v>1.834</v>
-      </c>
-    </row>
-    <row r="135" spans="1:2">
+        <v>1.8340000000000001</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>134</v>
       </c>
@@ -1813,15 +2025,15 @@
         <v>1.204</v>
       </c>
     </row>
-    <row r="136" spans="1:2">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>135</v>
       </c>
       <c r="B136">
-        <v>2.138</v>
-      </c>
-    </row>
-    <row r="137" spans="1:2">
+        <v>2.1379999999999999</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>136</v>
       </c>
@@ -1829,7 +2041,7 @@
         <v>2.177</v>
       </c>
     </row>
-    <row r="138" spans="1:2">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>137</v>
       </c>
@@ -1837,39 +2049,39 @@
         <v>1.91</v>
       </c>
     </row>
-    <row r="139" spans="1:2">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>138</v>
       </c>
       <c r="B139">
-        <v>2.348</v>
-      </c>
-    </row>
-    <row r="140" spans="1:2">
+        <v>2.3479999999999999</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>139</v>
       </c>
       <c r="B140">
-        <v>1.594</v>
-      </c>
-    </row>
-    <row r="141" spans="1:2">
+        <v>1.5940000000000001</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>140</v>
       </c>
       <c r="B141">
-        <v>2.244</v>
-      </c>
-    </row>
-    <row r="142" spans="1:2">
+        <v>2.2440000000000002</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>141</v>
       </c>
       <c r="B142">
-        <v>2.445</v>
-      </c>
-    </row>
-    <row r="143" spans="1:2">
+        <v>2.4449999999999998</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>142</v>
       </c>
@@ -1877,7 +2089,7 @@
         <v>2.57</v>
       </c>
     </row>
-    <row r="144" spans="1:2">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>143</v>
       </c>
@@ -1885,39 +2097,39 @@
         <v>2.734</v>
       </c>
     </row>
-    <row r="145" spans="1:2">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>144</v>
       </c>
       <c r="B145">
-        <v>2.336</v>
-      </c>
-    </row>
-    <row r="146" spans="1:2">
+        <v>2.3359999999999999</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>145</v>
       </c>
       <c r="B146">
-        <v>2.374</v>
-      </c>
-    </row>
-    <row r="147" spans="1:2">
+        <v>2.3740000000000001</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>146</v>
       </c>
       <c r="B147">
-        <v>2.082</v>
-      </c>
-    </row>
-    <row r="148" spans="1:2">
+        <v>2.0819999999999999</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>147</v>
       </c>
       <c r="B148">
-        <v>1.866</v>
-      </c>
-    </row>
-    <row r="149" spans="1:2">
+        <v>1.8660000000000001</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>148</v>
       </c>
@@ -1925,23 +2137,23 @@
         <v>2.706</v>
       </c>
     </row>
-    <row r="150" spans="1:2">
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>149</v>
       </c>
       <c r="B150">
-        <v>3.301</v>
-      </c>
-    </row>
-    <row r="151" spans="1:2">
+        <v>3.3010000000000002</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>150</v>
       </c>
       <c r="B151">
-        <v>2.517</v>
-      </c>
-    </row>
-    <row r="152" spans="1:2">
+        <v>2.5169999999999999</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>151</v>
       </c>
@@ -1949,7 +2161,7 @@
         <v>5.04</v>
       </c>
     </row>
-    <row r="153" spans="1:2">
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>152</v>
       </c>
@@ -1957,63 +2169,63 @@
         <v>2.544</v>
       </c>
     </row>
-    <row r="154" spans="1:2">
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>153</v>
       </c>
       <c r="B154">
-        <v>2.814</v>
-      </c>
-    </row>
-    <row r="155" spans="1:2">
+        <v>2.8140000000000001</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>154</v>
       </c>
       <c r="B155">
-        <v>2.906</v>
-      </c>
-    </row>
-    <row r="156" spans="1:2">
+        <v>2.9060000000000001</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>155</v>
       </c>
       <c r="B156">
-        <v>3.124</v>
-      </c>
-    </row>
-    <row r="157" spans="1:2">
+        <v>3.1240000000000001</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>156</v>
       </c>
       <c r="B157">
-        <v>3.292</v>
-      </c>
-    </row>
-    <row r="158" spans="1:2">
+        <v>3.2919999999999998</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>157</v>
       </c>
       <c r="B158">
-        <v>3.292</v>
-      </c>
-    </row>
-    <row r="159" spans="1:2">
+        <v>3.2919999999999998</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>158</v>
       </c>
       <c r="B159">
-        <v>3.885</v>
-      </c>
-    </row>
-    <row r="160" spans="1:2">
+        <v>3.8849999999999998</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>159</v>
       </c>
       <c r="B160">
-        <v>2.475</v>
-      </c>
-    </row>
-    <row r="161" spans="1:2">
+        <v>2.4750000000000001</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>160</v>
       </c>
@@ -2021,79 +2233,79 @@
         <v>2.274</v>
       </c>
     </row>
-    <row r="162" spans="1:2">
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>161</v>
       </c>
       <c r="B162">
-        <v>2.475</v>
-      </c>
-    </row>
-    <row r="163" spans="1:2">
+        <v>2.4750000000000001</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>162</v>
       </c>
       <c r="B163">
-        <v>2.974</v>
-      </c>
-    </row>
-    <row r="164" spans="1:2">
+        <v>2.9740000000000002</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>163</v>
       </c>
       <c r="B164">
-        <v>2.436</v>
-      </c>
-    </row>
-    <row r="165" spans="1:2">
+        <v>2.4359999999999999</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>164</v>
       </c>
       <c r="B165">
-        <v>2.481</v>
-      </c>
-    </row>
-    <row r="166" spans="1:2">
+        <v>2.4809999999999999</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>165</v>
       </c>
       <c r="B166">
-        <v>1.995</v>
-      </c>
-    </row>
-    <row r="167" spans="1:2">
+        <v>1.9950000000000001</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>166</v>
       </c>
       <c r="B167">
-        <v>2.526</v>
-      </c>
-    </row>
-    <row r="168" spans="1:2">
+        <v>2.5259999999999998</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>167</v>
       </c>
       <c r="B168">
-        <v>2.696</v>
-      </c>
-    </row>
-    <row r="169" spans="1:2">
+        <v>2.6960000000000002</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>168</v>
       </c>
       <c r="B169">
-        <v>2.795</v>
-      </c>
-    </row>
-    <row r="170" spans="1:2">
+        <v>2.7949999999999999</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>169</v>
       </c>
       <c r="B170">
-        <v>2.481</v>
-      </c>
-    </row>
-    <row r="171" spans="1:2">
+        <v>2.4809999999999999</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>170</v>
       </c>
@@ -2101,119 +2313,119 @@
         <v>2.819</v>
       </c>
     </row>
-    <row r="172" spans="1:2">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>171</v>
       </c>
       <c r="B172">
-        <v>1.965</v>
-      </c>
-    </row>
-    <row r="173" spans="1:2">
+        <v>1.9650000000000001</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>172</v>
       </c>
       <c r="B173">
-        <v>2.463</v>
-      </c>
-    </row>
-    <row r="174" spans="1:2">
+        <v>2.4630000000000001</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>173</v>
       </c>
       <c r="B174">
-        <v>2.414</v>
-      </c>
-    </row>
-    <row r="175" spans="1:2">
+        <v>2.4140000000000001</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>174</v>
       </c>
       <c r="B175">
-        <v>2.526</v>
-      </c>
-    </row>
-    <row r="176" spans="1:2">
+        <v>2.5259999999999998</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>175</v>
       </c>
       <c r="B176">
-        <v>2.021</v>
-      </c>
-    </row>
-    <row r="177" spans="1:2">
+        <v>2.0209999999999999</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>176</v>
       </c>
       <c r="B177">
-        <v>3.217</v>
-      </c>
-    </row>
-    <row r="178" spans="1:2">
+        <v>3.2170000000000001</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>177</v>
       </c>
       <c r="B178">
-        <v>2.861</v>
-      </c>
-    </row>
-    <row r="179" spans="1:2">
+        <v>2.8610000000000002</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>178</v>
       </c>
       <c r="B179">
-        <v>3.186</v>
-      </c>
-    </row>
-    <row r="180" spans="1:2">
+        <v>3.1859999999999999</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>179</v>
       </c>
       <c r="B180">
-        <v>2.463</v>
-      </c>
-    </row>
-    <row r="181" spans="1:2">
+        <v>2.4630000000000001</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>180</v>
       </c>
       <c r="B181">
-        <v>2.029</v>
-      </c>
-    </row>
-    <row r="182" spans="1:2">
+        <v>2.0289999999999999</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>181</v>
       </c>
       <c r="B182">
-        <v>2.209</v>
-      </c>
-    </row>
-    <row r="183" spans="1:2">
+        <v>2.2090000000000001</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>182</v>
       </c>
       <c r="B183">
-        <v>2.688</v>
-      </c>
-    </row>
-    <row r="184" spans="1:2">
+        <v>2.6880000000000002</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>183</v>
       </c>
       <c r="B184">
-        <v>2.574</v>
-      </c>
-    </row>
-    <row r="185" spans="1:2">
+        <v>2.5739999999999998</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>184</v>
       </c>
       <c r="B185">
-        <v>3.309</v>
-      </c>
-    </row>
-    <row r="186" spans="1:2">
+        <v>3.3090000000000002</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>185</v>
       </c>
@@ -2221,55 +2433,55 @@
         <v>2.14</v>
       </c>
     </row>
-    <row r="187" spans="1:2">
+    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>186</v>
       </c>
       <c r="B187">
-        <v>2.526</v>
-      </c>
-    </row>
-    <row r="188" spans="1:2">
+        <v>2.5259999999999998</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>187</v>
       </c>
       <c r="B188">
-        <v>2.526</v>
-      </c>
-    </row>
-    <row r="189" spans="1:2">
+        <v>2.5259999999999998</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>188</v>
       </c>
       <c r="B189">
-        <v>3.451</v>
-      </c>
-    </row>
-    <row r="190" spans="1:2">
+        <v>3.4510000000000001</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>189</v>
       </c>
       <c r="B190">
-        <v>2.574</v>
-      </c>
-    </row>
-    <row r="191" spans="1:2">
+        <v>2.5739999999999998</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>190</v>
       </c>
       <c r="B191">
-        <v>2.699</v>
-      </c>
-    </row>
-    <row r="192" spans="1:2">
+        <v>2.6989999999999998</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>191</v>
       </c>
       <c r="B192">
-        <v>2.526</v>
-      </c>
-    </row>
-    <row r="193" spans="1:2">
+        <v>2.5259999999999998</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>192</v>
       </c>
@@ -2277,7 +2489,7 @@
         <v>2.819</v>
       </c>
     </row>
-    <row r="194" spans="1:2">
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>193</v>
       </c>
@@ -2285,7 +2497,7 @@
         <v>2.754</v>
       </c>
     </row>
-    <row r="195" spans="1:2">
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>194</v>
       </c>
@@ -2293,15 +2505,15 @@
         <v>3.032</v>
       </c>
     </row>
-    <row r="196" spans="1:2">
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>195</v>
       </c>
       <c r="B196">
-        <v>1.918</v>
-      </c>
-    </row>
-    <row r="197" spans="1:2">
+        <v>1.9179999999999999</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>196</v>
       </c>
@@ -2309,23 +2521,23 @@
         <v>1.516</v>
       </c>
     </row>
-    <row r="198" spans="1:2">
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>197</v>
       </c>
       <c r="B198">
-        <v>3.451</v>
-      </c>
-    </row>
-    <row r="199" spans="1:2">
+        <v>3.4510000000000001</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>198</v>
       </c>
       <c r="B199">
-        <v>3.064</v>
-      </c>
-    </row>
-    <row r="200" spans="1:2">
+        <v>3.0640000000000001</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>199</v>
       </c>
@@ -2333,23 +2545,23 @@
         <v>2.597</v>
       </c>
     </row>
-    <row r="201" spans="1:2">
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>200</v>
       </c>
       <c r="B201">
-        <v>2.523</v>
-      </c>
-    </row>
-    <row r="202" spans="1:2">
+        <v>2.5230000000000001</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>201</v>
       </c>
       <c r="B202">
-        <v>2.26</v>
-      </c>
-    </row>
-    <row r="203" spans="1:2">
+        <v>2.2599999999999998</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>202</v>
       </c>
@@ -2357,39 +2569,39 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="204" spans="1:2">
+    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>203</v>
       </c>
       <c r="B204">
-        <v>2.341</v>
-      </c>
-    </row>
-    <row r="205" spans="1:2">
+        <v>2.3410000000000002</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>204</v>
       </c>
       <c r="B205">
-        <v>2.884</v>
-      </c>
-    </row>
-    <row r="206" spans="1:2">
+        <v>2.8839999999999999</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>205</v>
       </c>
       <c r="B206">
-        <v>2.451</v>
-      </c>
-    </row>
-    <row r="207" spans="1:2">
+        <v>2.4510000000000001</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>206</v>
       </c>
       <c r="B207">
-        <v>2.526</v>
-      </c>
-    </row>
-    <row r="208" spans="1:2">
+        <v>2.5259999999999998</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>207</v>
       </c>
@@ -2397,23 +2609,23 @@
         <v>2.206</v>
       </c>
     </row>
-    <row r="209" spans="1:2">
+    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>208</v>
       </c>
       <c r="B209">
-        <v>2.021</v>
-      </c>
-    </row>
-    <row r="210" spans="1:2">
+        <v>2.0209999999999999</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>209</v>
       </c>
       <c r="B210">
-        <v>1.965</v>
-      </c>
-    </row>
-    <row r="211" spans="1:2">
+        <v>1.9650000000000001</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A211">
         <v>210</v>
       </c>
@@ -2421,39 +2633,39 @@
         <v>3.39</v>
       </c>
     </row>
-    <row r="212" spans="1:2">
+    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A212">
         <v>211</v>
       </c>
       <c r="B212">
-        <v>2.094</v>
-      </c>
-    </row>
-    <row r="213" spans="1:2">
+        <v>2.0939999999999999</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A213">
         <v>212</v>
       </c>
       <c r="B213">
-        <v>2.795</v>
-      </c>
-    </row>
-    <row r="214" spans="1:2">
+        <v>2.7949999999999999</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A214">
         <v>213</v>
       </c>
       <c r="B214">
-        <v>2.696</v>
-      </c>
-    </row>
-    <row r="215" spans="1:2">
+        <v>2.6960000000000002</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A215">
         <v>214</v>
       </c>
       <c r="B215">
-        <v>2.312</v>
-      </c>
-    </row>
-    <row r="216" spans="1:2">
+        <v>2.3119999999999998</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A216">
         <v>215</v>
       </c>
@@ -2461,23 +2673,23 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="217" spans="1:2">
+    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A217">
         <v>216</v>
       </c>
       <c r="B217">
-        <v>2.354</v>
-      </c>
-    </row>
-    <row r="218" spans="1:2">
+        <v>2.3540000000000001</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A218">
         <v>217</v>
       </c>
       <c r="B218">
-        <v>2.951</v>
-      </c>
-    </row>
-    <row r="219" spans="1:2">
+        <v>2.9510000000000001</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>218</v>
       </c>
@@ -2485,15 +2697,15 @@
         <v>2.585</v>
       </c>
     </row>
-    <row r="220" spans="1:2">
+    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A220">
         <v>219</v>
       </c>
       <c r="B220">
-        <v>2.946</v>
-      </c>
-    </row>
-    <row r="221" spans="1:2">
+        <v>2.9460000000000002</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A221">
         <v>220</v>
       </c>
@@ -2501,7 +2713,7 @@
         <v>2.585</v>
       </c>
     </row>
-    <row r="222" spans="1:2">
+    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A222">
         <v>221</v>
       </c>
@@ -2509,7 +2721,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="223" spans="1:2">
+    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A223">
         <v>222</v>
       </c>
@@ -2517,7 +2729,7 @@
         <v>2.964</v>
       </c>
     </row>
-    <row r="224" spans="1:2">
+    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A224">
         <v>223</v>
       </c>
@@ -2525,15 +2737,15 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="225" spans="1:2">
+    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>224</v>
       </c>
       <c r="B225">
-        <v>2.209</v>
-      </c>
-    </row>
-    <row r="226" spans="1:2">
+        <v>2.2090000000000001</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A226">
         <v>225</v>
       </c>
@@ -2541,63 +2753,63 @@
         <v>1.516</v>
       </c>
     </row>
-    <row r="227" spans="1:2">
+    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A227">
         <v>226</v>
       </c>
       <c r="B227">
-        <v>2.108</v>
-      </c>
-    </row>
-    <row r="228" spans="1:2">
+        <v>2.1080000000000001</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A228">
         <v>227</v>
       </c>
       <c r="B228">
-        <v>3.179</v>
-      </c>
-    </row>
-    <row r="229" spans="1:2">
+        <v>3.1789999999999998</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A229">
         <v>228</v>
       </c>
       <c r="B229">
-        <v>1.598</v>
-      </c>
-    </row>
-    <row r="230" spans="1:2">
+        <v>1.5980000000000001</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A230">
         <v>229</v>
       </c>
       <c r="B230">
-        <v>2.526</v>
-      </c>
-    </row>
-    <row r="231" spans="1:2">
+        <v>2.5259999999999998</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A231">
         <v>230</v>
       </c>
       <c r="B231">
-        <v>3.365</v>
-      </c>
-    </row>
-    <row r="232" spans="1:2">
+        <v>3.3650000000000002</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A232">
         <v>231</v>
       </c>
       <c r="B232">
-        <v>2.28</v>
-      </c>
-    </row>
-    <row r="233" spans="1:2">
+        <v>2.2799999999999998</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A233">
         <v>232</v>
       </c>
       <c r="B233">
-        <v>2.144</v>
-      </c>
-    </row>
-    <row r="234" spans="1:2">
+        <v>2.1440000000000001</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A234">
         <v>233</v>
       </c>
@@ -2605,23 +2817,23 @@
         <v>2.964</v>
       </c>
     </row>
-    <row r="235" spans="1:2">
+    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A235">
         <v>234</v>
       </c>
       <c r="B235">
-        <v>2.523</v>
-      </c>
-    </row>
-    <row r="236" spans="1:2">
+        <v>2.5230000000000001</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A236">
         <v>235</v>
       </c>
       <c r="B236">
-        <v>3.817</v>
-      </c>
-    </row>
-    <row r="237" spans="1:2">
+        <v>3.8170000000000002</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A237">
         <v>236</v>
       </c>
@@ -2629,15 +2841,15 @@
         <v>3.032</v>
       </c>
     </row>
-    <row r="238" spans="1:2">
+    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A238">
         <v>237</v>
       </c>
       <c r="B238">
-        <v>2.696</v>
-      </c>
-    </row>
-    <row r="239" spans="1:2">
+        <v>2.6960000000000002</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A239">
         <v>238</v>
       </c>
@@ -2645,47 +2857,47 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="240" spans="1:2">
+    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A240">
         <v>239</v>
       </c>
       <c r="B240">
-        <v>2.631</v>
-      </c>
-    </row>
-    <row r="241" spans="1:2">
+        <v>2.6309999999999998</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A241">
         <v>240</v>
       </c>
       <c r="B241">
-        <v>2.962</v>
-      </c>
-    </row>
-    <row r="242" spans="1:2">
+        <v>2.9620000000000002</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A242">
         <v>241</v>
       </c>
       <c r="B242">
-        <v>3.179</v>
-      </c>
-    </row>
-    <row r="243" spans="1:2">
+        <v>3.1789999999999998</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A243">
         <v>242</v>
       </c>
       <c r="B243">
-        <v>2.821</v>
-      </c>
-    </row>
-    <row r="244" spans="1:2">
+        <v>2.8210000000000002</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A244">
         <v>243</v>
       </c>
       <c r="B244">
-        <v>2.26</v>
-      </c>
-    </row>
-    <row r="245" spans="1:2">
+        <v>2.2599999999999998</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A245">
         <v>244</v>
       </c>
@@ -2693,7 +2905,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="246" spans="1:2">
+    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A246">
         <v>245</v>
       </c>
@@ -2701,23 +2913,23 @@
         <v>3.347</v>
       </c>
     </row>
-    <row r="247" spans="1:2">
+    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A247">
         <v>246</v>
       </c>
       <c r="B247">
-        <v>2.795</v>
-      </c>
-    </row>
-    <row r="248" spans="1:2">
+        <v>2.7949999999999999</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A248">
         <v>247</v>
       </c>
       <c r="B248">
-        <v>2.526</v>
-      </c>
-    </row>
-    <row r="249" spans="1:2">
+        <v>2.5259999999999998</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A249">
         <v>248</v>
       </c>
@@ -2725,23 +2937,23 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="250" spans="1:2">
+    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A250">
         <v>249</v>
       </c>
       <c r="B250">
-        <v>2.481</v>
-      </c>
-    </row>
-    <row r="251" spans="1:2">
+        <v>2.4809999999999999</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A251">
         <v>250</v>
       </c>
       <c r="B251">
-        <v>1.965</v>
-      </c>
-    </row>
-    <row r="252" spans="1:2">
+        <v>1.9650000000000001</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A252">
         <v>251</v>
       </c>
@@ -2749,71 +2961,71 @@
         <v>2.379</v>
       </c>
     </row>
-    <row r="253" spans="1:2">
+    <row r="253" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A253">
         <v>252</v>
       </c>
       <c r="B253">
-        <v>2.357</v>
-      </c>
-    </row>
-    <row r="254" spans="1:2">
+        <v>2.3570000000000002</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A254">
         <v>253</v>
       </c>
       <c r="B254">
-        <v>1.733</v>
-      </c>
-    </row>
-    <row r="255" spans="1:2">
+        <v>1.7330000000000001</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A255">
         <v>254</v>
       </c>
       <c r="B255">
-        <v>2.209</v>
-      </c>
-    </row>
-    <row r="256" spans="1:2">
+        <v>2.2090000000000001</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A256">
         <v>255</v>
       </c>
       <c r="B256">
-        <v>3.064</v>
-      </c>
-    </row>
-    <row r="257" spans="1:2">
+        <v>3.0640000000000001</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A257">
         <v>256</v>
       </c>
       <c r="B257">
-        <v>2.951</v>
-      </c>
-    </row>
-    <row r="258" spans="1:2">
+        <v>2.9510000000000001</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A258">
         <v>257</v>
       </c>
       <c r="B258">
-        <v>3.537</v>
-      </c>
-    </row>
-    <row r="259" spans="1:2">
+        <v>3.5369999999999999</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A259">
         <v>258</v>
       </c>
       <c r="B259">
-        <v>2.029</v>
-      </c>
-    </row>
-    <row r="260" spans="1:2">
+        <v>2.0289999999999999</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A260">
         <v>259</v>
       </c>
       <c r="B260">
-        <v>2.054</v>
-      </c>
-    </row>
-    <row r="261" spans="1:2">
+        <v>2.0539999999999998</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A261">
         <v>260</v>
       </c>
@@ -2821,15 +3033,15 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="262" spans="1:2">
+    <row r="262" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A262">
         <v>261</v>
       </c>
       <c r="B262">
-        <v>2.209</v>
-      </c>
-    </row>
-    <row r="263" spans="1:2">
+        <v>2.2090000000000001</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A263">
         <v>262</v>
       </c>
@@ -2837,39 +3049,39 @@
         <v>2.14</v>
       </c>
     </row>
-    <row r="264" spans="1:2">
+    <row r="264" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A264">
         <v>263</v>
       </c>
       <c r="B264">
-        <v>2.094</v>
-      </c>
-    </row>
-    <row r="265" spans="1:2">
+        <v>2.0939999999999999</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A265">
         <v>264</v>
       </c>
       <c r="B265">
-        <v>2.861</v>
-      </c>
-    </row>
-    <row r="266" spans="1:2">
+        <v>2.8610000000000002</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A266">
         <v>265</v>
       </c>
       <c r="B266">
-        <v>3.687</v>
-      </c>
-    </row>
-    <row r="267" spans="1:2">
+        <v>3.6869999999999998</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A267">
         <v>266</v>
       </c>
       <c r="B267">
-        <v>2.172</v>
-      </c>
-    </row>
-    <row r="268" spans="1:2">
+        <v>2.1720000000000002</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A268">
         <v>267</v>
       </c>
@@ -2877,7 +3089,7 @@
         <v>2.379</v>
       </c>
     </row>
-    <row r="269" spans="1:2">
+    <row r="269" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A269">
         <v>268</v>
       </c>
@@ -2885,15 +3097,15 @@
         <v>2.984</v>
       </c>
     </row>
-    <row r="270" spans="1:2">
+    <row r="270" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A270">
         <v>269</v>
       </c>
       <c r="B270">
-        <v>2.289</v>
-      </c>
-    </row>
-    <row r="271" spans="1:2">
+        <v>2.2890000000000001</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A271">
         <v>270</v>
       </c>
@@ -2901,7 +3113,7 @@
         <v>3.347</v>
       </c>
     </row>
-    <row r="272" spans="1:2">
+    <row r="272" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A272">
         <v>271</v>
       </c>
@@ -2909,15 +3121,15 @@
         <v>1.855</v>
       </c>
     </row>
-    <row r="273" spans="1:2">
+    <row r="273" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A273">
         <v>272</v>
       </c>
       <c r="B273">
-        <v>2.869</v>
-      </c>
-    </row>
-    <row r="274" spans="1:2">
+        <v>2.8690000000000002</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A274">
         <v>273</v>
       </c>
@@ -2925,23 +3137,23 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="275" spans="1:2">
+    <row r="275" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A275">
         <v>274</v>
       </c>
       <c r="B275">
-        <v>2.773</v>
-      </c>
-    </row>
-    <row r="276" spans="1:2">
+        <v>2.7730000000000001</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A276">
         <v>275</v>
       </c>
       <c r="B276">
-        <v>1.938</v>
-      </c>
-    </row>
-    <row r="277" spans="1:2">
+        <v>1.9379999999999999</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A277">
         <v>276</v>
       </c>
@@ -2949,7 +3161,7 @@
         <v>3.004</v>
       </c>
     </row>
-    <row r="278" spans="1:2">
+    <row r="278" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A278">
         <v>277</v>
       </c>
@@ -2957,7 +3169,7 @@
         <v>3.004</v>
       </c>
     </row>
-    <row r="279" spans="1:2">
+    <row r="279" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A279">
         <v>278</v>
       </c>
@@ -2965,15 +3177,15 @@
         <v>2.645</v>
       </c>
     </row>
-    <row r="280" spans="1:2">
+    <row r="280" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A280">
         <v>279</v>
       </c>
       <c r="B280">
-        <v>2.054</v>
-      </c>
-    </row>
-    <row r="281" spans="1:2">
+        <v>2.0539999999999998</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A281">
         <v>280</v>
       </c>
@@ -2981,23 +3193,23 @@
         <v>3.238</v>
       </c>
     </row>
-    <row r="282" spans="1:2">
+    <row r="282" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A282">
         <v>281</v>
       </c>
       <c r="B282">
-        <v>2.442</v>
-      </c>
-    </row>
-    <row r="283" spans="1:2">
+        <v>2.4420000000000002</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A283">
         <v>282</v>
       </c>
       <c r="B283">
-        <v>1.938</v>
-      </c>
-    </row>
-    <row r="284" spans="1:2">
+        <v>1.9379999999999999</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A284">
         <v>283</v>
       </c>
@@ -3005,7 +3217,7 @@
         <v>1.976</v>
       </c>
     </row>
-    <row r="285" spans="1:2">
+    <row r="285" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A285">
         <v>284</v>
       </c>
@@ -3013,47 +3225,47 @@
         <v>1.867</v>
       </c>
     </row>
-    <row r="286" spans="1:2">
+    <row r="286" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A286">
         <v>285</v>
       </c>
       <c r="B286">
-        <v>2.463</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2">
+        <v>2.4630000000000001</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A287">
         <v>286</v>
       </c>
       <c r="B287">
-        <v>3.709</v>
-      </c>
-    </row>
-    <row r="288" spans="1:2">
+        <v>3.7090000000000001</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A288">
         <v>287</v>
       </c>
       <c r="B288">
-        <v>3.922</v>
-      </c>
-    </row>
-    <row r="289" spans="1:2">
+        <v>3.9220000000000002</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A289">
         <v>288</v>
       </c>
       <c r="B289">
-        <v>3.103</v>
-      </c>
-    </row>
-    <row r="290" spans="1:2">
+        <v>3.1030000000000002</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A290">
         <v>289</v>
       </c>
       <c r="B290">
-        <v>2.829</v>
-      </c>
-    </row>
-    <row r="291" spans="1:2">
+        <v>2.8290000000000002</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A291">
         <v>290</v>
       </c>
@@ -3061,23 +3273,23 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="292" spans="1:2">
+    <row r="292" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A292">
         <v>291</v>
       </c>
       <c r="B292">
-        <v>3.807</v>
-      </c>
-    </row>
-    <row r="293" spans="1:2">
+        <v>3.8069999999999999</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A293">
         <v>292</v>
       </c>
       <c r="B293">
-        <v>2.26</v>
-      </c>
-    </row>
-    <row r="294" spans="1:2">
+        <v>2.2599999999999998</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A294">
         <v>293</v>
       </c>
@@ -3085,15 +3297,15 @@
         <v>1.871</v>
       </c>
     </row>
-    <row r="295" spans="1:2">
+    <row r="295" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A295">
         <v>294</v>
       </c>
       <c r="B295">
-        <v>2.526</v>
-      </c>
-    </row>
-    <row r="296" spans="1:2">
+        <v>2.5259999999999998</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A296">
         <v>295</v>
       </c>
@@ -3101,44 +3313,44 @@
         <v>2.367</v>
       </c>
     </row>
-    <row r="297" spans="1:2">
+    <row r="297" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A297">
         <v>296</v>
       </c>
       <c r="B297">
-        <v>3.735</v>
-      </c>
-    </row>
-    <row r="298" spans="1:2">
+        <v>3.7349999999999999</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A298">
         <v>297</v>
       </c>
       <c r="B298">
-        <v>2.55</v>
-      </c>
-    </row>
-    <row r="299" spans="1:2">
+        <v>2.5499999999999998</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A299">
         <v>298</v>
       </c>
       <c r="B299">
-        <v>2.253</v>
-      </c>
-    </row>
-    <row r="300" spans="1:2">
+        <v>2.2530000000000001</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A300">
         <v>299</v>
       </c>
       <c r="B300">
-        <v>2.526</v>
-      </c>
-    </row>
-    <row r="301" spans="1:2">
+        <v>2.5259999999999998</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A301">
         <v>300</v>
       </c>
       <c r="B301">
-        <v>2.451</v>
+        <v>2.4510000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>